<commit_message>
New Spearman's rank correlation coefficient
</commit_message>
<xml_diff>
--- a/2VAR_ATSBR_T2W/2var_atsbr_t2w_BICYCLE.xlsx
+++ b/2VAR_ATSBR_T2W/2var_atsbr_t2w_BICYCLE.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11003"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/philliao/Downloads/Code/IB-Math-IA/2VAR_ATSBR_T2W/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38F72E0C-0D8A-AC4B-A90A-BD0AAF83A940}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDAA8286-99DA-324D-9A21-541CF55CE7DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="25600" windowHeight="14320" xr2:uid="{4D1AF13A-A5F1-E34F-94D2-60D62824593C}"/>
+    <workbookView xWindow="3840" yWindow="660" windowWidth="21760" windowHeight="14320" xr2:uid="{4D1AF13A-A5F1-E34F-94D2-60D62824593C}"/>
   </bookViews>
   <sheets>
     <sheet name="Regression" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="32">
   <si>
     <t>district_name</t>
   </si>
@@ -53,12 +53,93 @@
   <si>
     <t>r value</t>
   </si>
+  <si>
+    <t>SUMMARY OUTPUT</t>
+  </si>
+  <si>
+    <t>Regression Statistics</t>
+  </si>
+  <si>
+    <t>Multiple R</t>
+  </si>
+  <si>
+    <t>R Square</t>
+  </si>
+  <si>
+    <t>Adjusted R Square</t>
+  </si>
+  <si>
+    <t>Standard Error</t>
+  </si>
+  <si>
+    <t>Observations</t>
+  </si>
+  <si>
+    <t>ANOVA</t>
+  </si>
+  <si>
+    <t>Regression</t>
+  </si>
+  <si>
+    <t>Residual</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>Intercept</t>
+  </si>
+  <si>
+    <t>df</t>
+  </si>
+  <si>
+    <t>SS</t>
+  </si>
+  <si>
+    <t>MS</t>
+  </si>
+  <si>
+    <t>F</t>
+  </si>
+  <si>
+    <t>Significance F</t>
+  </si>
+  <si>
+    <t>Coefficients</t>
+  </si>
+  <si>
+    <t>t Stat</t>
+  </si>
+  <si>
+    <t>P-value</t>
+  </si>
+  <si>
+    <t>Lower 95%</t>
+  </si>
+  <si>
+    <t>Upper 95%</t>
+  </si>
+  <si>
+    <t>Lower 95.0%</t>
+  </si>
+  <si>
+    <t>Upper 95.0%</t>
+  </si>
+  <si>
+    <t>speed_acr_rank</t>
+  </si>
+  <si>
+    <t>Percent BICYCLE rank</t>
+  </si>
+  <si>
+    <t>rho=</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -85,6 +166,21 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -94,7 +190,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -102,18 +198,49 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="centerContinuous"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -163,13 +290,8 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US"/>
-              <a:t>Congestion Rate to Bicycle</a:t>
+              <a:t>ATSBR BICYCLE</a:t>
             </a:r>
-            <a:r>
-              <a:rPr lang="en-US" baseline="0"/>
-              <a:t> Rate</a:t>
-            </a:r>
-            <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:rich>
       </c:tx>
@@ -629,6 +751,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -636,7 +759,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -1136,6 +1258,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -1143,7 +1266,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -1213,11 +1335,11 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US"/>
-              <a:t>Congestion Rate to Bicycle</a:t>
+              <a:t>ATSBR BICYCLE</a:t>
             </a:r>
             <a:r>
               <a:rPr lang="en-US" baseline="0"/>
-              <a:t> Rate (Populated)</a:t>
+              <a:t> (Crowded)</a:t>
             </a:r>
             <a:endParaRPr lang="en-US"/>
           </a:p>
@@ -1649,6 +1771,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -1656,7 +1779,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -3795,8 +3917,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C79C884C-E453-6B44-ADBD-205B6FE17472}">
-  <dimension ref="A1:AN13"/>
+  <dimension ref="A1:AO50"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="45" max="45" width="14.1640625" customWidth="1"/>
+    <col min="46" max="46" width="15.1640625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
@@ -3932,6 +4058,10 @@
       </c>
       <c r="C5" s="3">
         <v>3.186801</v>
+      </c>
+      <c r="L5">
+        <f>CORREL(B2:B13, C2:C13)</f>
+        <v>0.59436329575376301</v>
       </c>
       <c r="O5" s="1">
         <v>4</v>
@@ -4137,8 +4267,1283 @@
       <c r="AD13" s="1"/>
       <c r="AE13" s="3"/>
     </row>
+    <row r="18" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A18" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E18" t="s">
+        <v>5</v>
+      </c>
+      <c r="O18" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="P18" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="Q18" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="S18" t="s">
+        <v>5</v>
+      </c>
+      <c r="AC18" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="AD18" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="AE18" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="AG18" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="19" spans="1:38" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="1">
+        <v>1</v>
+      </c>
+      <c r="B19" s="1">
+        <v>-8.9864000000000003E-3</v>
+      </c>
+      <c r="C19" s="3">
+        <v>15.58724</v>
+      </c>
+      <c r="O19" s="1">
+        <v>3</v>
+      </c>
+      <c r="P19" s="1">
+        <v>1.909891E-2</v>
+      </c>
+      <c r="Q19" s="3">
+        <v>28.346050000000002</v>
+      </c>
+      <c r="AC19" s="1">
+        <v>1</v>
+      </c>
+      <c r="AD19" s="1">
+        <v>-8.9864000000000003E-3</v>
+      </c>
+      <c r="AE19" s="3">
+        <v>15.58724</v>
+      </c>
+    </row>
+    <row r="20" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A20" s="1">
+        <v>2</v>
+      </c>
+      <c r="B20" s="1">
+        <v>-7.0763999999999994E-2</v>
+      </c>
+      <c r="C20" s="3">
+        <v>0.52957699999999996</v>
+      </c>
+      <c r="E20" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F20" s="6"/>
+      <c r="O20" s="1">
+        <v>4</v>
+      </c>
+      <c r="P20" s="1">
+        <v>3.064716E-2</v>
+      </c>
+      <c r="Q20" s="3">
+        <v>3.186801</v>
+      </c>
+      <c r="S20" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="T20" s="6"/>
+      <c r="AC20" s="1">
+        <v>2</v>
+      </c>
+      <c r="AD20" s="1">
+        <v>-7.0763999999999994E-2</v>
+      </c>
+      <c r="AE20" s="3">
+        <v>0.52957699999999996</v>
+      </c>
+      <c r="AG20" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="AH20" s="6"/>
+    </row>
+    <row r="21" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A21" s="1">
+        <v>3</v>
+      </c>
+      <c r="B21" s="1">
+        <v>1.909891E-2</v>
+      </c>
+      <c r="C21" s="3">
+        <v>28.346050000000002</v>
+      </c>
+      <c r="E21" t="s">
+        <v>7</v>
+      </c>
+      <c r="F21">
+        <v>0.59436329575376323</v>
+      </c>
+      <c r="O21" s="1">
+        <v>7</v>
+      </c>
+      <c r="P21" s="1">
+        <v>5.5768249999999998E-2</v>
+      </c>
+      <c r="Q21" s="3">
+        <v>33.591459999999998</v>
+      </c>
+      <c r="S21" t="s">
+        <v>7</v>
+      </c>
+      <c r="T21">
+        <v>0.49243635502324729</v>
+      </c>
+      <c r="AC21" s="1">
+        <v>5</v>
+      </c>
+      <c r="AD21" s="1">
+        <v>-1.3616899999999999E-2</v>
+      </c>
+      <c r="AE21" s="3">
+        <v>13.104430000000001</v>
+      </c>
+      <c r="AG21" t="s">
+        <v>7</v>
+      </c>
+      <c r="AH21">
+        <v>0.71377141225435903</v>
+      </c>
+    </row>
+    <row r="22" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A22" s="1">
+        <v>4</v>
+      </c>
+      <c r="B22" s="1">
+        <v>3.064716E-2</v>
+      </c>
+      <c r="C22" s="3">
+        <v>3.186801</v>
+      </c>
+      <c r="E22" t="s">
+        <v>8</v>
+      </c>
+      <c r="F22">
+        <v>0.35326772733927542</v>
+      </c>
+      <c r="O22" s="1">
+        <v>8</v>
+      </c>
+      <c r="P22" s="1">
+        <v>1.93241E-2</v>
+      </c>
+      <c r="Q22" s="3">
+        <v>19.313939999999999</v>
+      </c>
+      <c r="S22" t="s">
+        <v>8</v>
+      </c>
+      <c r="T22">
+        <v>0.24249356374858166</v>
+      </c>
+      <c r="AC22" s="1">
+        <v>6</v>
+      </c>
+      <c r="AD22" s="1">
+        <v>8.6388100000000002E-3</v>
+      </c>
+      <c r="AE22" s="3">
+        <v>8.7025860000000002</v>
+      </c>
+      <c r="AG22" t="s">
+        <v>8</v>
+      </c>
+      <c r="AH22">
+        <v>0.50946962895158221</v>
+      </c>
+    </row>
+    <row r="23" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A23" s="1">
+        <v>5</v>
+      </c>
+      <c r="B23" s="1">
+        <v>-1.3616899999999999E-2</v>
+      </c>
+      <c r="C23" s="3">
+        <v>13.104430000000001</v>
+      </c>
+      <c r="E23" t="s">
+        <v>9</v>
+      </c>
+      <c r="F23">
+        <v>0.28140858593252827</v>
+      </c>
+      <c r="O23" s="1">
+        <v>11</v>
+      </c>
+      <c r="P23" s="1">
+        <v>3.3507639999999998E-2</v>
+      </c>
+      <c r="Q23" s="3">
+        <v>0.60503200000000001</v>
+      </c>
+      <c r="S23" t="s">
+        <v>9</v>
+      </c>
+      <c r="T23">
+        <v>5.311695468572708E-2</v>
+      </c>
+      <c r="AC23" s="1">
+        <v>10</v>
+      </c>
+      <c r="AD23" s="1">
+        <v>-7.7793000000000003E-3</v>
+      </c>
+      <c r="AE23" s="3">
+        <v>7.6024139999999996</v>
+      </c>
+      <c r="AG23" t="s">
+        <v>9</v>
+      </c>
+      <c r="AH23">
+        <v>0.34595950526877628</v>
+      </c>
+    </row>
+    <row r="24" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A24" s="1">
+        <v>6</v>
+      </c>
+      <c r="B24" s="1">
+        <v>8.6388100000000002E-3</v>
+      </c>
+      <c r="C24" s="3">
+        <v>8.7025860000000002</v>
+      </c>
+      <c r="E24" t="s">
+        <v>10</v>
+      </c>
+      <c r="F24">
+        <v>3.0615359356089718E-2</v>
+      </c>
+      <c r="O24" s="1">
+        <v>12</v>
+      </c>
+      <c r="P24" s="1">
+        <v>5.5304150000000003E-2</v>
+      </c>
+      <c r="Q24" s="3">
+        <v>39.211069999999999</v>
+      </c>
+      <c r="S24" t="s">
+        <v>10</v>
+      </c>
+      <c r="T24">
+        <v>1.6054985739418808E-2</v>
+      </c>
+      <c r="AG24" t="s">
+        <v>10</v>
+      </c>
+      <c r="AH24">
+        <v>2.4587607701454097E-2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:38" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="1">
+        <v>7</v>
+      </c>
+      <c r="B25" s="1">
+        <v>5.5768249999999998E-2</v>
+      </c>
+      <c r="C25" s="3">
+        <v>33.591459999999998</v>
+      </c>
+      <c r="E25" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F25" s="4">
+        <v>11</v>
+      </c>
+      <c r="S25" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="T25" s="4">
+        <v>6</v>
+      </c>
+      <c r="AC25" s="1"/>
+      <c r="AD25" s="1"/>
+      <c r="AE25" s="3"/>
+      <c r="AG25" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="AH25" s="4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="26" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A26" s="1">
+        <v>8</v>
+      </c>
+      <c r="B26" s="1">
+        <v>1.93241E-2</v>
+      </c>
+      <c r="C26" s="3">
+        <v>19.313939999999999</v>
+      </c>
+      <c r="AC26" s="1"/>
+      <c r="AD26" s="1"/>
+      <c r="AE26" s="3"/>
+    </row>
+    <row r="27" spans="1:38" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="1">
+        <v>10</v>
+      </c>
+      <c r="B27" s="1">
+        <v>-7.7793000000000003E-3</v>
+      </c>
+      <c r="C27" s="3">
+        <v>7.6024139999999996</v>
+      </c>
+      <c r="E27" t="s">
+        <v>12</v>
+      </c>
+      <c r="O27" s="1"/>
+      <c r="P27" s="1"/>
+      <c r="S27" t="s">
+        <v>12</v>
+      </c>
+      <c r="AC27" s="1"/>
+      <c r="AD27" s="1"/>
+      <c r="AG27" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="28" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A28" s="1">
+        <v>11</v>
+      </c>
+      <c r="B28" s="1">
+        <v>3.3507639999999998E-2</v>
+      </c>
+      <c r="C28" s="3">
+        <v>0.60503200000000001</v>
+      </c>
+      <c r="E28" s="5"/>
+      <c r="F28" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="G28" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="H28" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="I28" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="J28" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="O28" s="1"/>
+      <c r="P28" s="1"/>
+      <c r="Q28" s="3"/>
+      <c r="S28" s="5"/>
+      <c r="T28" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="U28" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="V28" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="W28" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="X28" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="AG28" s="5"/>
+      <c r="AH28" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="AI28" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="AJ28" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="AK28" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="AL28" s="5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="29" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A29" s="1">
+        <v>12</v>
+      </c>
+      <c r="B29" s="1">
+        <v>5.5304150000000003E-2</v>
+      </c>
+      <c r="C29" s="3">
+        <v>39.211069999999999</v>
+      </c>
+      <c r="E29" t="s">
+        <v>13</v>
+      </c>
+      <c r="F29">
+        <v>1</v>
+      </c>
+      <c r="G29">
+        <v>4.6078747265212265E-3</v>
+      </c>
+      <c r="H29">
+        <v>4.6078747265212265E-3</v>
+      </c>
+      <c r="I29">
+        <v>4.9161139476974816</v>
+      </c>
+      <c r="J29" s="7">
+        <v>5.380663339245028E-2</v>
+      </c>
+      <c r="S29" t="s">
+        <v>13</v>
+      </c>
+      <c r="T29">
+        <v>1</v>
+      </c>
+      <c r="U29">
+        <v>3.3006063317251818E-4</v>
+      </c>
+      <c r="V29">
+        <v>3.3006063317251818E-4</v>
+      </c>
+      <c r="W29">
+        <v>1.2804831861156487</v>
+      </c>
+      <c r="X29" s="7">
+        <v>0.32105179078960383</v>
+      </c>
+      <c r="AC29" s="1"/>
+      <c r="AD29" s="1"/>
+      <c r="AE29" s="3"/>
+      <c r="AG29" t="s">
+        <v>13</v>
+      </c>
+      <c r="AH29">
+        <v>1</v>
+      </c>
+      <c r="AI29">
+        <v>1.883675993697465E-3</v>
+      </c>
+      <c r="AJ29">
+        <v>1.883675993697465E-3</v>
+      </c>
+      <c r="AK29">
+        <v>3.1158292677944806</v>
+      </c>
+      <c r="AL29" s="7">
+        <v>0.17571829360851857</v>
+      </c>
+    </row>
+    <row r="30" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="E30" t="s">
+        <v>14</v>
+      </c>
+      <c r="F30">
+        <v>9</v>
+      </c>
+      <c r="G30">
+        <v>8.4357020565225919E-3</v>
+      </c>
+      <c r="H30">
+        <v>9.3730022850251017E-4</v>
+      </c>
+      <c r="S30" t="s">
+        <v>14</v>
+      </c>
+      <c r="T30">
+        <v>4</v>
+      </c>
+      <c r="U30">
+        <v>1.0310502683717653E-3</v>
+      </c>
+      <c r="V30">
+        <v>2.5776256709294132E-4</v>
+      </c>
+      <c r="AC30" s="1"/>
+      <c r="AD30" s="1"/>
+      <c r="AE30" s="3"/>
+      <c r="AG30" t="s">
+        <v>14</v>
+      </c>
+      <c r="AH30">
+        <v>3</v>
+      </c>
+      <c r="AI30">
+        <v>1.8136513574418148E-3</v>
+      </c>
+      <c r="AJ30">
+        <v>6.0455045248060488E-4</v>
+      </c>
+    </row>
+    <row r="31" spans="1:38" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="E31" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F31" s="4">
+        <v>10</v>
+      </c>
+      <c r="G31" s="4">
+        <v>1.3043576783043818E-2</v>
+      </c>
+      <c r="H31" s="4"/>
+      <c r="I31" s="4"/>
+      <c r="J31" s="4"/>
+      <c r="S31" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="T31" s="4">
+        <v>5</v>
+      </c>
+      <c r="U31" s="4">
+        <v>1.3611109015442835E-3</v>
+      </c>
+      <c r="V31" s="4"/>
+      <c r="W31" s="4"/>
+      <c r="X31" s="4"/>
+      <c r="AG31" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="AH31" s="4">
+        <v>4</v>
+      </c>
+      <c r="AI31" s="4">
+        <v>3.6973273511392798E-3</v>
+      </c>
+      <c r="AJ31" s="4"/>
+      <c r="AK31" s="4"/>
+      <c r="AL31" s="4"/>
+    </row>
+    <row r="32" spans="1:38" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
+    <row r="33" spans="1:41" x14ac:dyDescent="0.2">
+      <c r="E33" s="5"/>
+      <c r="F33" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="G33" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="H33" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="I33" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="J33" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="K33" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="L33" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="M33" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="S33" s="5"/>
+      <c r="T33" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="U33" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="V33" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="W33" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="X33" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="Y33" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="Z33" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA33" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="AG33" s="5"/>
+      <c r="AH33" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="AI33" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="AJ33" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="AK33" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="AL33" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="AM33" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="AN33" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="AO33" s="5" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="34" spans="1:41" x14ac:dyDescent="0.2">
+      <c r="E34" t="s">
+        <v>16</v>
+      </c>
+      <c r="F34">
+        <v>-1.3813819279383233E-2</v>
+      </c>
+      <c r="G34">
+        <v>1.4511590468943231E-2</v>
+      </c>
+      <c r="H34">
+        <v>-0.9519162843622605</v>
+      </c>
+      <c r="I34" s="7">
+        <v>0.3660025689815003</v>
+      </c>
+      <c r="J34">
+        <v>-4.6641317602297332E-2</v>
+      </c>
+      <c r="K34">
+        <v>1.9013679043530865E-2</v>
+      </c>
+      <c r="L34">
+        <v>-4.6641317602297332E-2</v>
+      </c>
+      <c r="M34">
+        <v>1.9013679043530865E-2</v>
+      </c>
+      <c r="S34" t="s">
+        <v>16</v>
+      </c>
+      <c r="T34">
+        <v>2.5091309491970859E-2</v>
+      </c>
+      <c r="U34">
+        <v>1.1372806675756757E-2</v>
+      </c>
+      <c r="V34">
+        <v>2.2062548153093671</v>
+      </c>
+      <c r="W34" s="7">
+        <v>9.200908470892552E-2</v>
+      </c>
+      <c r="X34">
+        <v>-6.4846639352947773E-3</v>
+      </c>
+      <c r="Y34">
+        <v>5.6667282919236499E-2</v>
+      </c>
+      <c r="Z34">
+        <v>-6.4846639352947773E-3</v>
+      </c>
+      <c r="AA34">
+        <v>5.6667282919236499E-2</v>
+      </c>
+      <c r="AG34" t="s">
+        <v>16</v>
+      </c>
+      <c r="AH34">
+        <v>-5.2643418750208469E-2</v>
+      </c>
+      <c r="AI34">
+        <v>2.2249074134465818E-2</v>
+      </c>
+      <c r="AJ34">
+        <v>-2.366094806105171</v>
+      </c>
+      <c r="AK34" s="7">
+        <v>9.8852692995067742E-2</v>
+      </c>
+      <c r="AL34">
+        <v>-0.12344990252542255</v>
+      </c>
+      <c r="AM34">
+        <v>1.8163065025005611E-2</v>
+      </c>
+      <c r="AN34">
+        <v>-0.12344990252542255</v>
+      </c>
+      <c r="AO34">
+        <v>1.8163065025005611E-2</v>
+      </c>
+    </row>
+    <row r="35" spans="1:41" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="E35" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="F35" s="4">
+        <v>1.6085137646657836E-3</v>
+      </c>
+      <c r="G35" s="4">
+        <v>7.2546056766717329E-4</v>
+      </c>
+      <c r="H35" s="4">
+        <v>2.2172311444000323</v>
+      </c>
+      <c r="I35" s="8">
+        <v>5.3806633392450377E-2</v>
+      </c>
+      <c r="J35" s="4">
+        <v>-3.2592054810164581E-5</v>
+      </c>
+      <c r="K35" s="4">
+        <v>3.249619584141732E-3</v>
+      </c>
+      <c r="L35" s="4">
+        <v>-3.2592054810164581E-5</v>
+      </c>
+      <c r="M35" s="4">
+        <v>3.249619584141732E-3</v>
+      </c>
+      <c r="S35" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="T35" s="4">
+        <v>5.0784822844938732E-4</v>
+      </c>
+      <c r="U35" s="4">
+        <v>4.4879395825464313E-4</v>
+      </c>
+      <c r="V35" s="4">
+        <v>1.1315843698618535</v>
+      </c>
+      <c r="W35" s="8">
+        <v>0.32105179078960377</v>
+      </c>
+      <c r="X35" s="4">
+        <v>-7.3820356018905941E-4</v>
+      </c>
+      <c r="Y35" s="4">
+        <v>1.753900017087834E-3</v>
+      </c>
+      <c r="Z35" s="4">
+        <v>-7.3820356018905941E-4</v>
+      </c>
+      <c r="AA35" s="4">
+        <v>1.753900017087834E-3</v>
+      </c>
+      <c r="AG35" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="AH35" s="4">
+        <v>3.7496897943518678E-3</v>
+      </c>
+      <c r="AI35" s="4">
+        <v>2.1242641240850719E-3</v>
+      </c>
+      <c r="AJ35" s="4">
+        <v>1.7651711723780452</v>
+      </c>
+      <c r="AK35" s="8">
+        <v>0.17571829360851851</v>
+      </c>
+      <c r="AL35" s="4">
+        <v>-3.0106667187894038E-3</v>
+      </c>
+      <c r="AM35" s="4">
+        <v>1.0510046307493139E-2</v>
+      </c>
+      <c r="AN35" s="4">
+        <v>-3.0106667187894038E-3</v>
+      </c>
+      <c r="AO35" s="4">
+        <v>1.0510046307493139E-2</v>
+      </c>
+    </row>
+    <row r="39" spans="1:41" x14ac:dyDescent="0.2">
+      <c r="A39" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E39" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="O39" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="P39" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="Q39" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="R39" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="S39" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="AC39" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="AD39" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="AE39" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="AF39" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="AG39" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="40" spans="1:41" x14ac:dyDescent="0.2">
+      <c r="A40" s="1">
+        <v>1</v>
+      </c>
+      <c r="B40" s="1">
+        <v>-8.9864000000000003E-3</v>
+      </c>
+      <c r="C40">
+        <f t="shared" ref="C40:C50" si="0">_xlfn.RANK.AVG(B40,B$40:B$50,1)</f>
+        <v>3</v>
+      </c>
+      <c r="D40" s="3">
+        <v>15.58724</v>
+      </c>
+      <c r="E40">
+        <f t="shared" ref="E40:E50" si="1">_xlfn.RANK.AVG(D40,D$40:D$50,1)</f>
+        <v>7</v>
+      </c>
+      <c r="O40" s="1">
+        <v>3</v>
+      </c>
+      <c r="P40" s="1">
+        <v>1.909891E-2</v>
+      </c>
+      <c r="Q40">
+        <f t="shared" ref="Q40:Q45" si="2">_xlfn.RANK.AVG(P40, P$40:P$45, 1)</f>
+        <v>1</v>
+      </c>
+      <c r="R40" s="3">
+        <v>28.346050000000002</v>
+      </c>
+      <c r="S40">
+        <f t="shared" ref="S40:S45" si="3">_xlfn.RANK.AVG(R40, R$40:R$45, 1)</f>
+        <v>4</v>
+      </c>
+      <c r="AC40" s="1">
+        <v>1</v>
+      </c>
+      <c r="AD40" s="1">
+        <v>-8.9864000000000003E-3</v>
+      </c>
+      <c r="AE40">
+        <f>_xlfn.RANK.AVG(AD40, AD$40:AD$44, 1)</f>
+        <v>3</v>
+      </c>
+      <c r="AF40" s="3">
+        <v>15.58724</v>
+      </c>
+      <c r="AG40">
+        <f>_xlfn.RANK.AVG(AF40, AF$40:AF$44, 1)</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="41" spans="1:41" x14ac:dyDescent="0.2">
+      <c r="A41" s="1">
+        <v>2</v>
+      </c>
+      <c r="B41" s="1">
+        <v>-7.0763999999999994E-2</v>
+      </c>
+      <c r="C41">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+      <c r="D41" s="3">
+        <v>0.52957699999999996</v>
+      </c>
+      <c r="E41">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="G41" t="s">
+        <v>31</v>
+      </c>
+      <c r="H41">
+        <f>CORREL(C40:C50,E40:E50)</f>
+        <v>0.46363636363636357</v>
+      </c>
+      <c r="O41" s="1">
+        <v>4</v>
+      </c>
+      <c r="P41" s="1">
+        <v>3.064716E-2</v>
+      </c>
+      <c r="Q41">
+        <f t="shared" si="2"/>
+        <v>3</v>
+      </c>
+      <c r="R41" s="3">
+        <v>3.186801</v>
+      </c>
+      <c r="S41">
+        <f t="shared" si="3"/>
+        <v>2</v>
+      </c>
+      <c r="U41" t="s">
+        <v>31</v>
+      </c>
+      <c r="V41">
+        <f>CORREL(Q40:Q45,S40:S45)</f>
+        <v>0.37142857142857144</v>
+      </c>
+      <c r="AC41" s="1">
+        <v>2</v>
+      </c>
+      <c r="AD41" s="1">
+        <v>-7.0763999999999994E-2</v>
+      </c>
+      <c r="AE41">
+        <f>_xlfn.RANK.AVG(AD41, AD$40:AD$44, 1)</f>
+        <v>1</v>
+      </c>
+      <c r="AF41" s="3">
+        <v>0.52957699999999996</v>
+      </c>
+      <c r="AG41">
+        <f>_xlfn.RANK.AVG(AF41, AF$40:AF$44, 1)</f>
+        <v>1</v>
+      </c>
+      <c r="AI41" t="s">
+        <v>31</v>
+      </c>
+      <c r="AJ41">
+        <f>CORREL(AE40:AE44,AG40:AG44)</f>
+        <v>0.19999999999999996</v>
+      </c>
+    </row>
+    <row r="42" spans="1:41" x14ac:dyDescent="0.2">
+      <c r="A42" s="1">
+        <v>3</v>
+      </c>
+      <c r="B42" s="1">
+        <v>1.909891E-2</v>
+      </c>
+      <c r="C42">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="D42" s="3">
+        <v>28.346050000000002</v>
+      </c>
+      <c r="E42">
+        <f t="shared" si="1"/>
+        <v>9</v>
+      </c>
+      <c r="O42" s="1">
+        <v>7</v>
+      </c>
+      <c r="P42" s="1">
+        <v>5.5768249999999998E-2</v>
+      </c>
+      <c r="Q42">
+        <f t="shared" si="2"/>
+        <v>6</v>
+      </c>
+      <c r="R42" s="3">
+        <v>33.591459999999998</v>
+      </c>
+      <c r="S42">
+        <f t="shared" si="3"/>
+        <v>5</v>
+      </c>
+      <c r="AC42" s="1">
+        <v>5</v>
+      </c>
+      <c r="AD42" s="1">
+        <v>-1.3616899999999999E-2</v>
+      </c>
+      <c r="AE42">
+        <f>_xlfn.RANK.AVG(AD42, AD$40:AD$44, 1)</f>
+        <v>2</v>
+      </c>
+      <c r="AF42" s="3">
+        <v>13.104430000000001</v>
+      </c>
+      <c r="AG42">
+        <f>_xlfn.RANK.AVG(AF42, AF$40:AF$44, 1)</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="43" spans="1:41" x14ac:dyDescent="0.2">
+      <c r="A43" s="1">
+        <v>4</v>
+      </c>
+      <c r="B43" s="1">
+        <v>3.064716E-2</v>
+      </c>
+      <c r="C43">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+      <c r="D43" s="3">
+        <v>3.186801</v>
+      </c>
+      <c r="E43">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="O43" s="1">
+        <v>8</v>
+      </c>
+      <c r="P43" s="1">
+        <v>1.93241E-2</v>
+      </c>
+      <c r="Q43">
+        <f t="shared" si="2"/>
+        <v>2</v>
+      </c>
+      <c r="R43" s="3">
+        <v>19.313939999999999</v>
+      </c>
+      <c r="S43">
+        <f t="shared" si="3"/>
+        <v>3</v>
+      </c>
+      <c r="AC43" s="1">
+        <v>6</v>
+      </c>
+      <c r="AD43" s="1">
+        <v>8.6388100000000002E-3</v>
+      </c>
+      <c r="AE43">
+        <f>_xlfn.RANK.AVG(AD43, AD$40:AD$44, 1)</f>
+        <v>5</v>
+      </c>
+      <c r="AF43" s="3">
+        <v>8.7025860000000002</v>
+      </c>
+      <c r="AG43">
+        <f>_xlfn.RANK.AVG(AF43, AF$40:AF$44, 1)</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="44" spans="1:41" x14ac:dyDescent="0.2">
+      <c r="A44" s="1">
+        <v>5</v>
+      </c>
+      <c r="B44" s="1">
+        <v>-1.3616899999999999E-2</v>
+      </c>
+      <c r="C44">
+        <f t="shared" si="0"/>
+        <v>2</v>
+      </c>
+      <c r="D44" s="3">
+        <v>13.104430000000001</v>
+      </c>
+      <c r="E44">
+        <f t="shared" si="1"/>
+        <v>6</v>
+      </c>
+      <c r="O44" s="1">
+        <v>11</v>
+      </c>
+      <c r="P44" s="1">
+        <v>3.3507639999999998E-2</v>
+      </c>
+      <c r="Q44">
+        <f t="shared" si="2"/>
+        <v>4</v>
+      </c>
+      <c r="R44" s="3">
+        <v>0.60503200000000001</v>
+      </c>
+      <c r="S44">
+        <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="AC44" s="1">
+        <v>10</v>
+      </c>
+      <c r="AD44" s="1">
+        <v>-7.7793000000000003E-3</v>
+      </c>
+      <c r="AE44">
+        <f>_xlfn.RANK.AVG(AD44, AD$40:AD$44, 1)</f>
+        <v>4</v>
+      </c>
+      <c r="AF44" s="3">
+        <v>7.6024139999999996</v>
+      </c>
+      <c r="AG44">
+        <f>_xlfn.RANK.AVG(AF44, AF$40:AF$44, 1)</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="45" spans="1:41" x14ac:dyDescent="0.2">
+      <c r="A45" s="1">
+        <v>6</v>
+      </c>
+      <c r="B45" s="1">
+        <v>8.6388100000000002E-3</v>
+      </c>
+      <c r="C45">
+        <f t="shared" si="0"/>
+        <v>5</v>
+      </c>
+      <c r="D45" s="3">
+        <v>8.7025860000000002</v>
+      </c>
+      <c r="E45">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="O45" s="1">
+        <v>12</v>
+      </c>
+      <c r="P45" s="1">
+        <v>5.5304150000000003E-2</v>
+      </c>
+      <c r="Q45">
+        <f t="shared" si="2"/>
+        <v>5</v>
+      </c>
+      <c r="R45" s="3">
+        <v>39.211069999999999</v>
+      </c>
+      <c r="S45">
+        <f t="shared" si="3"/>
+        <v>6</v>
+      </c>
+    </row>
+    <row r="46" spans="1:41" x14ac:dyDescent="0.2">
+      <c r="A46" s="1">
+        <v>7</v>
+      </c>
+      <c r="B46" s="1">
+        <v>5.5768249999999998E-2</v>
+      </c>
+      <c r="C46">
+        <f t="shared" si="0"/>
+        <v>11</v>
+      </c>
+      <c r="D46" s="3">
+        <v>33.591459999999998</v>
+      </c>
+      <c r="E46">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="47" spans="1:41" x14ac:dyDescent="0.2">
+      <c r="A47" s="1">
+        <v>8</v>
+      </c>
+      <c r="B47" s="1">
+        <v>1.93241E-2</v>
+      </c>
+      <c r="C47">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="D47" s="3">
+        <v>19.313939999999999</v>
+      </c>
+      <c r="E47">
+        <f t="shared" si="1"/>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="48" spans="1:41" x14ac:dyDescent="0.2">
+      <c r="A48" s="1">
+        <v>10</v>
+      </c>
+      <c r="B48" s="1">
+        <v>-7.7793000000000003E-3</v>
+      </c>
+      <c r="C48">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="D48" s="3">
+        <v>7.6024139999999996</v>
+      </c>
+      <c r="E48">
+        <f t="shared" si="1"/>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A49" s="1">
+        <v>11</v>
+      </c>
+      <c r="B49" s="1">
+        <v>3.3507639999999998E-2</v>
+      </c>
+      <c r="C49">
+        <f t="shared" si="0"/>
+        <v>9</v>
+      </c>
+      <c r="D49" s="3">
+        <v>0.60503200000000001</v>
+      </c>
+      <c r="E49">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A50" s="1">
+        <v>12</v>
+      </c>
+      <c r="B50" s="1">
+        <v>5.5304150000000003E-2</v>
+      </c>
+      <c r="C50">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="D50" s="3">
+        <v>39.211069999999999</v>
+      </c>
+      <c r="E50">
+        <f t="shared" si="1"/>
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>

</xml_diff>